<commit_message>
feat: add LoCoMo and MEME benchmark support, improve experiment utilities
- Add LoCoMo benchmark loader (src/benchmark/locomo.py) with dialogue formatting
- Add LoCoMo-specific extract templates (Extract_Stage_LoCoMo.jinja,
  Extract_Stage_LoCoMo_Dense.jinja) and RD classify template
- Add LoCoMo memory extract schemas with evidence tracking
  (LoCoMoMemExtractResponse, normalize_extract_memories)
- Update extract_candidates.py for LoCoMo auto-detection and dialogue format
- Add config files for LoCoMo (default, dense_gran4, e4b, q35) and MEME bench
- Support attribute-based config path access in experiment_artifacts.py
- Update GPU/MAX_MODEL_LEN settings in model launch scripts
- Add MEME benchmark design docs and plan
- Add judge/eval scripts for tl1024 and direct judge runs
</commit_message>
<xml_diff>
--- a/results/experiment_results_all_methods_zjj.xlsx
+++ b/results/experiment_results_all_methods_zjj.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Sheet" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="tl256" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="tl512" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="tl1024" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -679,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1195,11 +1196,11 @@
           <t>gemma4-26B</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="8" t="n"/>
-      <c r="F27" s="8" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="20" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
@@ -1350,6 +1351,166 @@
       <c r="F33" s="28" t="inlineStr">
         <is>
           <t>RD (74.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Qwen3.5-4B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Filler</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>add_all</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>mem0</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>evermemos</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>N0</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>86.17</v>
+      </c>
+      <c r="C37" t="n">
+        <v>86.81</v>
+      </c>
+      <c r="D37" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="E37" t="n">
+        <v>86.81</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>add_all (86.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="C38" t="n">
+        <v>76.81</v>
+      </c>
+      <c r="D38" t="n">
+        <v>74.68000000000001</v>
+      </c>
+      <c r="E38" t="n">
+        <v>74.26000000000001</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>relation_decision (78.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>75.31999999999999</v>
+      </c>
+      <c r="C39" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="D39" t="n">
+        <v>67.66</v>
+      </c>
+      <c r="E39" t="n">
+        <v>47.02</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>relation_decision (75.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>70.43000000000001</v>
+      </c>
+      <c r="C40" t="n">
+        <v>25.74</v>
+      </c>
+      <c r="D40" t="n">
+        <v>61.91</v>
+      </c>
+      <c r="E40" t="n">
+        <v>36.81</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>relation_decision (70.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="C41" t="n">
+        <v>25.11</v>
+      </c>
+      <c r="D41" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="E41" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>relation_decision (66.81)</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1887,11 +2048,11 @@
           <t>gemma4-26B</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="8" t="n"/>
-      <c r="F27" s="8" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="20" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
@@ -2042,6 +2203,166 @@
       <c r="F33" s="28" t="inlineStr">
         <is>
           <t>RD (82.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Qwen3.5-4B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Filler</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>add_all</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>mem0</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>evermemos</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>N0</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="C37" t="n">
+        <v>87.45</v>
+      </c>
+      <c r="D37" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="E37" t="n">
+        <v>89.15000000000001</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>evermemos (89.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>84.68000000000001</v>
+      </c>
+      <c r="C38" t="n">
+        <v>85.53</v>
+      </c>
+      <c r="D38" t="n">
+        <v>81.48999999999999</v>
+      </c>
+      <c r="E38" t="n">
+        <v>86.81</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>evermemos (86.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>81.48999999999999</v>
+      </c>
+      <c r="C39" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="D39" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="E39" t="n">
+        <v>84.68000000000001</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>evermemos (84.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>81.48999999999999</v>
+      </c>
+      <c r="C40" t="n">
+        <v>81.06</v>
+      </c>
+      <c r="D40" t="n">
+        <v>80.20999999999999</v>
+      </c>
+      <c r="E40" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>relation_decision (81.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>82.34</v>
+      </c>
+      <c r="C41" t="n">
+        <v>67.87</v>
+      </c>
+      <c r="D41" t="n">
+        <v>79.36</v>
+      </c>
+      <c r="E41" t="n">
+        <v>61.91</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>relation_decision (82.34)</t>
         </is>
       </c>
     </row>
@@ -2055,4 +2376,343 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>LME Golden Memory — tl1024 (Judge: deepseek-v4-flash)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gemma4-e4b</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Filler</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>add_all</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>mem0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>evermemos</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>N0</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>86.59999999999999</v>
+      </c>
+      <c r="C5" t="n">
+        <v>88.09</v>
+      </c>
+      <c r="D5" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>89.56999999999999</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>evermemos (89.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="C6" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>65.31999999999999</v>
+      </c>
+      <c r="E6" t="n">
+        <v>85.31999999999999</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>relation_decision (85.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>85.11</v>
+      </c>
+      <c r="C7" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="D7" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="E7" t="n">
+        <v>83.83</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>relation_decision (85.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>84.68000000000001</v>
+      </c>
+      <c r="C8" t="n">
+        <v>84.04000000000001</v>
+      </c>
+      <c r="D8" t="n">
+        <v>63.62</v>
+      </c>
+      <c r="E8" t="n">
+        <v>84.68000000000001</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>relation_decision (84.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="C9" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="D9" t="n">
+        <v>60.43</v>
+      </c>
+      <c r="E9" t="n">
+        <v>82.98</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>add_all (83.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Qwen3.5-4B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Filler</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>add_all</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>mem0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>evermemos</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>N0</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="E13" t="n">
+        <v>87.23</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>relation_decision (88.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>85.53</v>
+      </c>
+      <c r="C14" t="n">
+        <v>86.38</v>
+      </c>
+      <c r="D14" t="n">
+        <v>79.79000000000001</v>
+      </c>
+      <c r="E14" t="n">
+        <v>85.53</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>add_all (86.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>82.77</v>
+      </c>
+      <c r="C15" t="n">
+        <v>84.26000000000001</v>
+      </c>
+      <c r="D15" t="n">
+        <v>80.43000000000001</v>
+      </c>
+      <c r="E15" t="n">
+        <v>85.31999999999999</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>evermemos (85.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>81.91</v>
+      </c>
+      <c r="C16" t="n">
+        <v>84.04000000000001</v>
+      </c>
+      <c r="D16" t="n">
+        <v>79.79000000000001</v>
+      </c>
+      <c r="E16" t="n">
+        <v>84.04000000000001</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>add_all (84.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>82.55</v>
+      </c>
+      <c r="C17" t="n">
+        <v>83.62</v>
+      </c>
+      <c r="D17" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="E17" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>add_all (83.62)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>